<commit_message>
batch mode render for fixed LOD issue
</commit_message>
<xml_diff>
--- a/data_output/segur_psd_fit_python/PSD_fit_results.xlsx
+++ b/data_output/segur_psd_fit_python/PSD_fit_results.xlsx
@@ -498,25 +498,25 @@
         <v>165</v>
       </c>
       <c r="C2" t="n">
-        <v>385</v>
+        <v>460</v>
       </c>
       <c r="D2" t="n">
-        <v>-1.919519209984631</v>
+        <v>-2.178262314101336</v>
       </c>
       <c r="E2" t="n">
-        <v>6.646352222023229</v>
+        <v>7.188966785993433</v>
       </c>
       <c r="F2" t="n">
-        <v>0.9880166882373123</v>
+        <v>0.9874272327052629</v>
       </c>
       <c r="G2" t="n">
-        <v>38</v>
+        <v>46</v>
       </c>
       <c r="H2" t="n">
-        <v>-2.919519209984631</v>
+        <v>-3.178262314101336</v>
       </c>
       <c r="I2" t="n">
-        <v>8502461.709674481</v>
+        <v>33657120.98314211</v>
       </c>
       <c r="J2" t="n">
         <v>1</v>
@@ -525,7 +525,7 @@
         <v>5000</v>
       </c>
       <c r="L2" t="n">
-        <v>4429474.313386698</v>
+        <v>15451362.52429571</v>
       </c>
       <c r="M2" t="n">
         <v>0</v>
@@ -543,28 +543,28 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>95</v>
+        <v>125</v>
       </c>
       <c r="C3" t="n">
-        <v>350</v>
+        <v>330</v>
       </c>
       <c r="D3" t="n">
-        <v>-2.739182076027633</v>
+        <v>-2.796397493529946</v>
       </c>
       <c r="E3" t="n">
-        <v>8.072532486656989</v>
+        <v>8.164359017622759</v>
       </c>
       <c r="F3" t="n">
-        <v>0.9929734699598479</v>
+        <v>0.9908877410115398</v>
       </c>
       <c r="G3" t="n">
-        <v>38</v>
+        <v>30</v>
       </c>
       <c r="H3" t="n">
-        <v>-3.739182076027633</v>
+        <v>-3.796397493529946</v>
       </c>
       <c r="I3" t="n">
-        <v>323707966.6876923</v>
+        <v>408279826.7525871</v>
       </c>
       <c r="J3" t="n">
         <v>1</v>
@@ -573,7 +573,7 @@
         <v>5000</v>
       </c>
       <c r="L3" t="n">
-        <v>118176870.9341352</v>
+        <v>146002071.4790114</v>
       </c>
       <c r="M3" t="n">
         <v>0</v>
@@ -591,28 +591,28 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>175</v>
+        <v>170</v>
       </c>
       <c r="C4" t="n">
         <v>480</v>
       </c>
       <c r="D4" t="n">
-        <v>-1.67106150944134</v>
+        <v>-1.735140565387896</v>
       </c>
       <c r="E4" t="n">
-        <v>5.896144627132704</v>
+        <v>5.961682977544652</v>
       </c>
       <c r="F4" t="n">
-        <v>0.9696822374227052</v>
+        <v>0.9608973398845442</v>
       </c>
       <c r="G4" t="n">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="H4" t="n">
-        <v>-2.671061509441341</v>
+        <v>-2.735140565387896</v>
       </c>
       <c r="I4" t="n">
-        <v>1315639.981915651</v>
+        <v>1588611.275448175</v>
       </c>
       <c r="J4" t="n">
         <v>1</v>
@@ -621,7 +621,7 @@
         <v>5000</v>
       </c>
       <c r="L4" t="n">
-        <v>787307.4136762404</v>
+        <v>915551.5701158018</v>
       </c>
       <c r="M4" t="n">
         <v>0</v>
@@ -645,22 +645,22 @@
         <v>560</v>
       </c>
       <c r="D5" t="n">
-        <v>-1.98298364129834</v>
+        <v>-1.969281003697001</v>
       </c>
       <c r="E5" t="n">
-        <v>6.848251205382933</v>
+        <v>6.794419287454688</v>
       </c>
       <c r="F5" t="n">
-        <v>0.9962128598531879</v>
+        <v>0.9944016755275872</v>
       </c>
       <c r="G5" t="n">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="H5" t="n">
-        <v>-2.98298364129834</v>
+        <v>-2.969281003697001</v>
       </c>
       <c r="I5" t="n">
-        <v>13982033.45297438</v>
+        <v>12266678.39068415</v>
       </c>
       <c r="J5" t="n">
         <v>1</v>
@@ -669,7 +669,7 @@
         <v>5000</v>
       </c>
       <c r="L5" t="n">
-        <v>7051007.640846008</v>
+        <v>6229013.396386933</v>
       </c>
       <c r="M5" t="n">
         <v>0</v>
@@ -693,22 +693,22 @@
         <v>410</v>
       </c>
       <c r="D6" t="n">
-        <v>-2.576619420139119</v>
+        <v>-2.537141017015231</v>
       </c>
       <c r="E6" t="n">
-        <v>7.932215013029039</v>
+        <v>7.810628033600369</v>
       </c>
       <c r="F6" t="n">
-        <v>0.9917455917646081</v>
+        <v>0.9923810700594311</v>
       </c>
       <c r="G6" t="n">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="H6" t="n">
-        <v>-3.576619420139119</v>
+        <v>-3.537141017015231</v>
       </c>
       <c r="I6" t="n">
-        <v>220427253.1853068</v>
+        <v>164048642.1557541</v>
       </c>
       <c r="J6" t="n">
         <v>1</v>
@@ -717,7 +717,7 @@
         <v>5000</v>
       </c>
       <c r="L6" t="n">
-        <v>85549014.8826395</v>
+        <v>64658858.52931897</v>
       </c>
       <c r="M6" t="n">
         <v>0</v>
@@ -741,22 +741,22 @@
         <v>585</v>
       </c>
       <c r="D7" t="n">
-        <v>-1.470704947074662</v>
+        <v>-1.468227363734859</v>
       </c>
       <c r="E7" t="n">
-        <v>5.363330702665392</v>
+        <v>5.347549482326052</v>
       </c>
       <c r="F7" t="n">
-        <v>0.9865468308222398</v>
+        <v>0.9876996299709244</v>
       </c>
       <c r="G7" t="n">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="H7" t="n">
-        <v>-2.470704947074662</v>
+        <v>-2.468227363734859</v>
       </c>
       <c r="I7" t="n">
-        <v>339512.8810262204</v>
+        <v>326845.7153969181</v>
       </c>
       <c r="J7" t="n">
         <v>1</v>
@@ -765,7 +765,7 @@
         <v>5000</v>
       </c>
       <c r="L7" t="n">
-        <v>230849.5998943134</v>
+        <v>222611.641573885</v>
       </c>
       <c r="M7" t="n">
         <v>0</v>
@@ -789,22 +789,22 @@
         <v>245</v>
       </c>
       <c r="D8" t="n">
-        <v>-1.765263164794791</v>
+        <v>-1.707671168080249</v>
       </c>
       <c r="E8" t="n">
-        <v>5.343845860830124</v>
+        <v>5.211815504510901</v>
       </c>
       <c r="F8" t="n">
-        <v>0.9939172884363451</v>
+        <v>0.9927208015648868</v>
       </c>
       <c r="G8" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="H8" t="n">
-        <v>-2.765263164794791</v>
+        <v>-2.70767116808025</v>
       </c>
       <c r="I8" t="n">
-        <v>389632.6298958096</v>
+        <v>278112.0142317772</v>
       </c>
       <c r="J8" t="n">
         <v>1</v>
@@ -813,7 +813,7 @@
         <v>5000</v>
       </c>
       <c r="L8" t="n">
-        <v>220722.0558307586</v>
+        <v>162860.3242115948</v>
       </c>
       <c r="M8" t="n">
         <v>0</v>
@@ -837,22 +837,22 @@
         <v>220</v>
       </c>
       <c r="D9" t="n">
-        <v>-2.15057100900288</v>
+        <v>-2.074025886910791</v>
       </c>
       <c r="E9" t="n">
-        <v>6.080429843520262</v>
+        <v>5.906229229854062</v>
       </c>
       <c r="F9" t="n">
-        <v>0.9946449592773108</v>
+        <v>0.9930485588491925</v>
       </c>
       <c r="G9" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="H9" t="n">
-        <v>-3.15057100900288</v>
+        <v>-3.074025886910791</v>
       </c>
       <c r="I9" t="n">
-        <v>2588115.361490024</v>
+        <v>1671257.628327265</v>
       </c>
       <c r="J9" t="n">
         <v>1</v>
@@ -861,7 +861,7 @@
         <v>5000</v>
       </c>
       <c r="L9" t="n">
-        <v>1203454.953099421</v>
+        <v>805803.6320993932</v>
       </c>
       <c r="M9" t="n">
         <v>0</v>

</xml_diff>